<commit_message>
Publish IG - 2026-08-03
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-actigraphy-metric-cs.xlsx
+++ b/docs/CodeSystem-actigraphy-metric-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.6.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-25T15:07:02-06:00</t>
+    <t>2026-08-03T22:31:50-05:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>